<commit_message>
docs: synchronize DS402 Home document set
</commit_message>
<xml_diff>
--- a/docs/api/API_DEVELOPMENT_PROGRESS.xlsx
+++ b/docs/api/API_DEVELOPMENT_PROGRESS.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R23fca56e7a964496"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API 현황" sheetId="2" r:id="R7956335447a94592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검증 현황" sheetId="3" r:id="Rac87b196b5d7487d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="우선순위" sheetId="4" r:id="R25a7f327d24b47de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R8d9429bdde154b5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API 현황" sheetId="2" r:id="R301886e5457a4582"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검증 현황" sheetId="3" r:id="R50052ad21b644e53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="우선순위" sheetId="4" r:id="Re4fe99a7ec284bcd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1114,7 +1114,7 @@
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>1.0-current | 2026-08-20 | LasalMotionControlLib 0.9.1-preview | production NO-GO</x:v>
+        <x:v>1.6-current | 2026-09-14 | LasalMotionControlLib 0.9.1-preview | production NO-GO</x:v>
       </x:c>
       <x:c r="B3" s="8" t="str">
         <x:v>1.0-current | 2026-08-20 | LasalMotionControlLib 0.9.1-preview | production NO-GO</x:v>
@@ -1140,7 +1140,7 @@
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="12" t="str">
-        <x:v>정본: docs/api/API_DEVELOPMENT_PROGRESS.md | SHA-256 83AAD3FC6876706421236AF083B212E06D67AC88D32A60493AFAAA9192B31F93 | 이 XLSX는 Markdown 정본에서 생성한 파생 산출물이며 직접 편집하지 않는다.</x:v>
+        <x:v>정본: docs/api/API_DEVELOPMENT_PROGRESS.md | SHA-256 62BFA2976BD0EF6D8DB99D56F1341423A600F436BB585E8C462BA4B0761C60FF | 이 XLSX는 Markdown 정본에서 생성한 파생 산출물이다.</x:v>
       </x:c>
       <x:c r="B4" s="12" t="str">
         <x:v>정본: docs/api/API_DEVELOPMENT_PROGRESS.md | SHA-256 236FDB65961701F0F3451B1F1295D1FADFB704BECCC6E1F1FC2881C869B28CF1 | 이 XLSX는 Markdown 정본에서 생성한 파생 산출물이며 직접 편집하지 않는다.</x:v>
@@ -1232,7 +1232,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="42" t="str">
-        <x:v>RELEASE STATUS: PRODUCTION NO-GO — current artifact identity drift로 UDP current gate 및 full SourceOnly가 STOP 상태</x:v>
+        <x:v>RELEASE STATUS: PRODUCTION NO-GO — DS402 Home 구현 완료와 Method 37 사용자 실기 확인은 moving method 및 전체 release PASS가 아님</x:v>
       </x:c>
       <x:c r="B10" s="42" t="str">
         <x:v>RELEASE STATUS: PRODUCTION NO-GO — current artifact identity drift로 UDP current gate 및 full SourceOnly가 STOP 상태</x:v>
@@ -1322,7 +1322,7 @@
         <x:v>Active</x:v>
       </x:c>
       <x:c r="G14" s="55" t="n">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="H14" s="55" t="str">
         <x:v>source-active / 기능별 적격성 상이</x:v>
@@ -1346,10 +1346,10 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G15" s="57" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H15" s="57" t="str">
-        <x:v>SetPosition, DS402 Home, SetOperationMode(PC/SDK)</x:v>
+        <x:v>SetPosition</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1366,7 +1366,7 @@
         <x:v>부분 구현 또는 제한 활성화</x:v>
       </x:c>
       <x:c r="F16" s="55" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Dormant</x:v>
       </x:c>
       <x:c r="G16" s="55" t="n">
         <x:v>1</x:v>
@@ -1854,16 +1854,16 @@
         <x:v>0x7D15/7D16/7D17</x:v>
       </x:c>
       <x:c r="C10" s="55" t="str">
-        <x:v>Dormant</x:v>
+        <x:v>Active/Limited</x:v>
       </x:c>
       <x:c r="D10" s="55" t="str">
-        <x:v>method37 source, gate FALSE, bit6 OFF</x:v>
+        <x:v>public LMC_HomeDS402 API; standard method/parameter 구현 완료; saved pre-Home mode 복귀</x:v>
       </x:c>
       <x:c r="E10" s="55" t="str">
-        <x:v>Source</x:v>
+        <x:v>Source + Method 37 user runtime</x:v>
       </x:c>
       <x:c r="F10" s="55" t="str">
-        <x:v>HomeDS402Ex execution + live proof</x:v>
+        <x:v>moving method 개별 실축 qualification</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="45" customHeight="1">
@@ -2592,6 +2592,29 @@
       </x:c>
       <x:c r="G18" s="61" t="str">
         <x:v>SetOpMode 11 tests</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="61" t="str">
+        <x:v>DS402 Home Method 37</x:v>
+      </x:c>
+      <x:c r="B19" s="61" t="str">
+        <x:v>사용자 정상 구동 확인</x:v>
+      </x:c>
+      <x:c r="C19" s="61" t="str">
+        <x:v>PASS/Limited</x:v>
+      </x:c>
+      <x:c r="D19" s="61" t="str">
+        <x:v>PLC runtime / physical</x:v>
+      </x:c>
+      <x:c r="E19" s="61" t="str">
+        <x:v>Method 37 정상 구동</x:v>
+      </x:c>
+      <x:c r="F19" s="61" t="str">
+        <x:v>moving method 및 fault/restart/packet matrix 아님</x:v>
+      </x:c>
+      <x:c r="G19" s="61" t="str">
+        <x:v>2026-09-14 user evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2943,22 +2966,22 @@
     </x:row>
     <x:row r="14" ht="45" customHeight="1">
       <x:c r="A14" s="55" t="str">
-        <x:v>P3</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="B14" s="55" t="str">
-        <x:v>2.4 release semantic policy/generator/render 승격</x:v>
+        <x:v>DS402 Home moving method 개별 실축 검증</x:v>
       </x:c>
       <x:c r="C14" s="55" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="D14" s="55" t="str">
-        <x:v>policy tests + DOCX/PDF review</x:v>
+        <x:v>method별 switch/index, 방향, 종단, offset 및 saved-mode restore 확인</x:v>
       </x:c>
       <x:c r="E14" s="55" t="str">
-        <x:v>기존 2.3 배포본 덮어쓰기 금지</x:v>
+        <x:v>Method 37 PASS를 다른 method로 확대 금지</x:v>
       </x:c>
       <x:c r="F14" s="55" t="str">
-        <x:v>Distribution tooling</x:v>
+        <x:v>DS402 Home 2026-09-14 design/progress</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>